<commit_message>
Mock 5: round 1 marks of the second review in Cowork (58 good, 2 bad: M5-S33 and M5-S45). The owner did not mark. The assistant typed the marks on the instruction of the owner.
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TnghEw2ou31QVRW6aTsXeq
</commit_message>
<xml_diff>
--- a/marking/M5-round1.xlsx
+++ b/marking/M5-round1.xlsx
@@ -596,7 +596,11 @@
 D: The per-file passes fix the shallow analysis. Without a cross-file integration pass, however, nothing checks the data passed between files, so the mismatches stay hidden.</t>
         </is>
       </c>
-      <c r="N2" s="4" t="n"/>
+      <c r="N2" s="4" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="O2" s="4" t="n"/>
     </row>
     <row r="3">
@@ -669,7 +673,11 @@
 E: This keeps the long sequential wait and the three separate answers, so it skips parallel investigation with shared context and a unified synthesis.</t>
         </is>
       </c>
-      <c r="N3" s="4" t="n"/>
+      <c r="N3" s="4" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="O3" s="4" t="n"/>
     </row>
     <row r="4">
@@ -737,7 +745,11 @@
 D: The guide says to write tests before implementation. Tests generated from finished code only lock in existing defects and cannot guide improvement.</t>
         </is>
       </c>
-      <c r="N4" s="4" t="n"/>
+      <c r="N4" s="4" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="O4" s="4" t="n"/>
     </row>
     <row r="5">
@@ -805,7 +817,11 @@
 D: This puts the stale tool results back into the new context, which removes the advantage that a fresh session with a summary has over resuming with stale tool results.</t>
         </is>
       </c>
-      <c r="N5" s="4" t="n"/>
+      <c r="N5" s="4" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="O5" s="4" t="n"/>
     </row>
     <row r="6">
@@ -873,7 +889,11 @@
 D: The analyses are independent, so the passed findings save little work, and the subagents still run one after another across separate turns. The latency problem stays.</t>
         </is>
       </c>
-      <c r="N6" s="4" t="n"/>
+      <c r="N6" s="4" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="O6" s="4" t="n"/>
     </row>
     <row r="7">
@@ -941,7 +961,11 @@
 D: A prompt rule gives only probabilistic compliance, so the agent may still release to production without approval; the policy needs the deterministic guarantee of a hook.</t>
         </is>
       </c>
-      <c r="N7" s="4" t="n"/>
+      <c r="N7" s="4" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="O7" s="4" t="n"/>
     </row>
     <row r="8">
@@ -1009,7 +1033,11 @@
 D: The guide describes a prioritized plan that adapts as dependencies are discovered; it does not call for discarding the existing map and plan after each new finding.</t>
         </is>
       </c>
-      <c r="N8" s="4" t="n"/>
+      <c r="N8" s="4" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="O8" s="4" t="n"/>
     </row>
     <row r="9">
@@ -1077,7 +1105,11 @@
 D: The imports of the defining file lead to its dependencies, not to its callers; the guide uses Grep to search content across the codebase for callers.</t>
         </is>
       </c>
-      <c r="N9" s="4" t="n"/>
+      <c r="N9" s="4" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="O9" s="4" t="n"/>
     </row>
     <row r="10">
@@ -1145,7 +1177,11 @@
 D: The guide names MCP resources as the mechanism for exposing content catalogs, such as documentation hierarchies and database schemas. They give the agent visibility into the available data without exploratory tool calls.</t>
         </is>
       </c>
-      <c r="N10" s="4" t="n"/>
+      <c r="N10" s="4" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="O10" s="4" t="n"/>
     </row>
     <row r="11">
@@ -1213,7 +1249,11 @@
 D: The max_tokens limit caps the length of the generated output and does not decide which tool the model selects. The reliability drop follows the growth from 5 to 21 tools.</t>
         </is>
       </c>
-      <c r="N11" s="4" t="n"/>
+      <c r="N11" s="4" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="O11" s="4" t="n"/>
     </row>
     <row r="12">
@@ -1281,7 +1321,11 @@
 D: The guide says loop control should continue on "tool_use" and terminate on "end_turn". Checking for assistant text as a completion indicator is an anti-pattern.</t>
         </is>
       </c>
-      <c r="N12" s="4" t="n"/>
+      <c r="N12" s="4" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="O12" s="4" t="n"/>
     </row>
     <row r="13">
@@ -1349,7 +1393,11 @@
 D: The isError flag reports a failed tool call; it does not disconnect a server. The CI log tools were already available because all servers' tools are discovered at connection time.</t>
         </is>
       </c>
-      <c r="N13" s="4" t="n"/>
+      <c r="N13" s="4" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="O13" s="4" t="n"/>
     </row>
     <row r="14">
@@ -1417,7 +1465,11 @@
 D: The guide says that the session that generated code is less effective at reviewing its own changes than an independent review instance, and this change gives no list of already-posted findings.</t>
         </is>
       </c>
-      <c r="N14" s="4" t="n"/>
+      <c r="N14" s="4" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="O14" s="4" t="n"/>
     </row>
     <row r="15">
@@ -1490,7 +1542,11 @@
 E: The guide states that allowedTools must include "Task" for a coordinator to invoke subagents. The current list lacks it.</t>
         </is>
       </c>
-      <c r="N15" s="4" t="n"/>
+      <c r="N15" s="4" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="O15" s="4" t="n"/>
     </row>
     <row r="16">
@@ -1558,7 +1614,11 @@
 D: Glob only finds files by path pattern. The problem is a non-unique match inside one file, so Edit fails again for the same reason.</t>
         </is>
       </c>
-      <c r="N16" s="4" t="n"/>
+      <c r="N16" s="4" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="O16" s="4" t="n"/>
     </row>
     <row r="17">
@@ -1626,7 +1686,11 @@
 D: The guide states that plan mode enables safe codebase exploration and design before committing to changes, which prevents costly rework.</t>
         </is>
       </c>
-      <c r="N17" s="4" t="n"/>
+      <c r="N17" s="4" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="O17" s="4" t="n"/>
     </row>
     <row r="18">
@@ -1694,7 +1758,11 @@
 D: A multi-file change with multiple valid approaches calls for plan mode first. Deciding the approach during implementation risks costly rework.</t>
         </is>
       </c>
-      <c r="N18" s="4" t="n"/>
+      <c r="N18" s="4" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="O18" s="4" t="n"/>
     </row>
     <row r="19">
@@ -1762,7 +1830,11 @@
 D: This changes the configuration before diagnosing the cause, and it removes the package scoping that the directory-level hierarchy provides.</t>
         </is>
       </c>
-      <c r="N19" s="4" t="n"/>
+      <c r="N19" s="4" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="O19" s="4" t="n"/>
     </row>
     <row r="20">
@@ -1830,7 +1902,11 @@
 D: This edits the shared skill that teammates use, and context: fork only isolates skill output from the main conversation; it does not create a personal variant.</t>
         </is>
       </c>
-      <c r="N20" s="4" t="n"/>
+      <c r="N20" s="4" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="O20" s="4" t="n"/>
     </row>
     <row r="21">
@@ -1903,7 +1979,11 @@
 E: The guide says that summaries are injected into the initial context of the next-phase subagents, because those subagents receive only what their prompt gives them.</t>
         </is>
       </c>
-      <c r="N21" s="4" t="n"/>
+      <c r="N21" s="4" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="O21" s="4" t="n"/>
     </row>
     <row r="22">
@@ -1971,7 +2051,11 @@
 D: Plan mode lets a developer review the approach before execution. It does not change how the synthesis step merges records, so the extra sources are still lost.</t>
         </is>
       </c>
-      <c r="N22" s="4" t="n"/>
+      <c r="N22" s="4" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="O22" s="4" t="n"/>
     </row>
     <row r="23">
@@ -2039,7 +2123,11 @@
 D: This treats an access failure (a timeout) as a valid empty result, which the guide says must be kept distinct so that the right decision can be made.</t>
         </is>
       </c>
-      <c r="N23" s="4" t="n"/>
+      <c r="N23" s="4" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="O23" s="4" t="n"/>
     </row>
     <row r="24">
@@ -2112,7 +2200,11 @@
 E: The guide separates issues by whether their fixes interact, not by where tests live, and the discount fix interacts with the tax and formatter fixes.</t>
         </is>
       </c>
-      <c r="N24" s="4" t="n"/>
+      <c r="N24" s="4" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="O24" s="4" t="n"/>
     </row>
     <row r="25">
@@ -2180,7 +2272,11 @@
 D: Progressive summarization risks condensing numbers, dates, and stated expectations into vague summaries, which matches the vague wording that appeared after the /compact runs.</t>
         </is>
       </c>
-      <c r="N25" s="4" t="n"/>
+      <c r="N25" s="4" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="O25" s="4" t="n"/>
     </row>
     <row r="26">
@@ -2248,7 +2344,11 @@
 D: Context isolation keeps the main session clean but does not resolve which of several matching accounts is correct, so the guessing continues.</t>
         </is>
       </c>
-      <c r="N26" s="4" t="n"/>
+      <c r="N26" s="4" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="O26" s="4" t="n"/>
     </row>
     <row r="27">
@@ -2316,7 +2416,11 @@
 D: The guide warns that one aggregate accuracy figure can hide poor performance in specific segments. Stratifying the sample exists to show the error rate of each segment.</t>
         </is>
       </c>
-      <c r="N27" s="4" t="n"/>
+      <c r="N27" s="4" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="O27" s="4" t="n"/>
     </row>
     <row r="28">
@@ -2384,7 +2488,11 @@
 D: The guide warns that an aggregate figure can mask poor performance in a specific segment, and here it hides 72% accuracy on the Java authentication field.</t>
         </is>
       </c>
-      <c r="N28" s="4" t="n"/>
+      <c r="N28" s="4" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="O28" s="4" t="n"/>
     </row>
     <row r="29">
@@ -2452,7 +2560,11 @@
 D: The guide presents claim-source mappings as the way to preserve attribution through synthesis. A mapping can show both values with their sources, so it does not force one source per claim.</t>
         </is>
       </c>
-      <c r="N29" s="4" t="n"/>
+      <c r="N29" s="4" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="O29" s="4" t="n"/>
     </row>
     <row r="30">
@@ -2520,7 +2632,11 @@
 D: The guide names a date validation conditional as a simple, well-scoped change for direct execution. It has no verbose discovery that could exhaust the context.</t>
         </is>
       </c>
-      <c r="N30" s="4" t="n"/>
+      <c r="N30" s="4" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="O30" s="4" t="n"/>
     </row>
     <row r="31">
@@ -2588,7 +2704,11 @@
 D: The @import syntax references an external file from CLAUDE.md, which keeps the configuration modular and includes only the standards that are relevant to the package.</t>
         </is>
       </c>
-      <c r="N31" s="4" t="n"/>
+      <c r="N31" s="4" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="O31" s="4" t="n"/>
     </row>
     <row r="32">
@@ -2661,7 +2781,11 @@
 E: With "auto" the model may return text instead of calling the tool, which loses guaranteed structured output and does nothing to normalize value formats.</t>
         </is>
       </c>
-      <c r="N32" s="4" t="n"/>
+      <c r="N32" s="4" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="O32" s="4" t="n"/>
     </row>
     <row r="33">
@@ -2729,7 +2853,11 @@
 D: The guide states that a detected_pattern field on structured findings tracks which code constructs trigger findings and enables analysis of false positive patterns when developers dismiss them.</t>
         </is>
       </c>
-      <c r="N33" s="4" t="n"/>
+      <c r="N33" s="4" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="O33" s="4" t="n"/>
     </row>
     <row r="34">
@@ -2797,8 +2925,16 @@
 D: The guide says that argument-hint prompts developers for required parameters, and this has no effect on which tools the skill can call.</t>
         </is>
       </c>
-      <c r="N34" s="4" t="n"/>
-      <c r="O34" s="4" t="n"/>
+      <c r="N34" s="4" t="inlineStr">
+        <is>
+          <t>bad</t>
+        </is>
+      </c>
+      <c r="O34" s="4" t="inlineStr">
+        <is>
+          <t>Copy of M2-S34: a CI test-generation skill ran a Bash command that deleted a fixture directory, the answer is allowed-tools, and the three wrong options are the same (context: fork, argument-hint, a CLAUDE.md rule). Keep point 3.2-K2, but make a different frontmatter field the answer, for example context: fork or argument-hint.</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
@@ -2865,7 +3001,11 @@
 D: Schema-enforced structured output gives schema-compliant output and eliminates syntax errors; the findings carry valid defect values, so malformed strings are not the cause.</t>
         </is>
       </c>
-      <c r="N35" s="4" t="n"/>
+      <c r="N35" s="4" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="O35" s="4" t="n"/>
     </row>
     <row r="36">
@@ -2933,7 +3073,11 @@
 D: Retries cannot recover information that is absent from the source, so the first group gets fabricated values, and the loop does not show how to read the table format.</t>
         </is>
       </c>
-      <c r="N36" s="4" t="n"/>
+      <c r="N36" s="4" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="O36" s="4" t="n"/>
     </row>
     <row r="37">
@@ -3001,7 +3145,11 @@
 D: The same specific error feedback fixed the misnamed fields, and no error message can make Claude Code produce criteria that are absent from its input.</t>
         </is>
       </c>
-      <c r="N37" s="4" t="n"/>
+      <c r="N37" s="4" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="O37" s="4" t="n"/>
     </row>
     <row r="38">
@@ -3069,7 +3217,11 @@
 D: The root CLAUDE.md loads in every session, so the data-retention conventions add irrelevant context for all other services. A heading does not make them load conditionally.</t>
         </is>
       </c>
-      <c r="N38" s="4" t="n"/>
+      <c r="N38" s="4" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="O38" s="4" t="n"/>
     </row>
     <row r="39">
@@ -3142,7 +3294,11 @@
 E: The missing latency SLA in the guide concerns when results arrive. These requests failed because they exceeded the context limit, and that limit is unrelated to waiting time.</t>
         </is>
       </c>
-      <c r="N39" s="4" t="n"/>
+      <c r="N39" s="4" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="O39" s="4" t="n"/>
     </row>
     <row r="40">
@@ -3210,7 +3366,11 @@
 D: Finding volume is not the cause of the lost trust, so the noisy naming-convention category keeps undermining trust and accurate security findings are lost.</t>
         </is>
       </c>
-      <c r="N40" s="4" t="n"/>
+      <c r="N40" s="4" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="O40" s="4" t="n"/>
     </row>
     <row r="41">
@@ -3278,7 +3438,11 @@
 D: The guide says explicit severity criteria with concrete code examples for each severity level achieve consistent classification.</t>
         </is>
       </c>
-      <c r="N41" s="4" t="n"/>
+      <c r="N41" s="4" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="O41" s="4" t="n"/>
     </row>
     <row r="42">
@@ -3346,7 +3510,11 @@
 D: A model keeps the reasoning context from generation, so in the same session it is less likely to question its own decisions. The fresh session has no such context, which explains why it finds the weak tests.</t>
         </is>
       </c>
-      <c r="N42" s="4" t="n"/>
+      <c r="N42" s="4" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="O42" s="4" t="n"/>
     </row>
     <row r="43">
@@ -3414,7 +3582,11 @@
 D: Documenting fixtures in CLAUDE.md improves test quality, and the team already does this; it does not tell Claude which scenarios the existing tests already check.</t>
         </is>
       </c>
-      <c r="N43" s="4" t="n"/>
+      <c r="N43" s="4" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="O43" s="4" t="n"/>
     </row>
     <row r="44">
@@ -3482,7 +3654,11 @@
 D: The guide describes custom_id as a field for correlating batch request and response pairs, not as a setting that controls processing priority.</t>
         </is>
       </c>
-      <c r="N44" s="4" t="n"/>
+      <c r="N44" s="4" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="O44" s="4" t="n"/>
     </row>
     <row r="45">
@@ -3550,7 +3726,11 @@
 D: The mismatches occur in small pull requests, so diff length does not explain why the flag is always false.</t>
         </is>
       </c>
-      <c r="N45" s="4" t="n"/>
+      <c r="N45" s="4" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="O45" s="4" t="n"/>
     </row>
     <row r="46">
@@ -3618,8 +3798,16 @@
 D: The guide uses per-file passes against attention dilution in large multi-file reviews. These pull requests touch only two or three files, and the uniform scores come from scoring in the session that produced the findings.</t>
         </is>
       </c>
-      <c r="N46" s="4" t="n"/>
-      <c r="O46" s="4" t="n"/>
+      <c r="N46" s="4" t="inlineStr">
+        <is>
+          <t>bad</t>
+        </is>
+      </c>
+      <c r="O46" s="4" t="inlineStr">
+        <is>
+          <t>Repeat of M5-S41 in the same scenario: both answers are 'the same session keeps its reasoning'. It also misses its point 4.6-S3. Keep the point. The answer must be about the verification pass that reports confidence so that findings can be routed for review. Do not use the same-session idea, and do not add a wrong option on self-reported confidence (scenario 5 already has one in M5-S40).</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
@@ -3686,7 +3874,11 @@
 D: This builds understanding incrementally. Grep finds the entry points, and Read then follows the imports to trace the flow, without loading all files upfront.</t>
         </is>
       </c>
-      <c r="N47" s="4" t="n"/>
+      <c r="N47" s="4" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="O47" s="4" t="n"/>
     </row>
     <row r="48">
@@ -3754,7 +3946,11 @@
 D: The agent never learns about the failure, so it cannot make a recovery decision; the guide says failures must be communicated back to the agent with the isError flag.</t>
         </is>
       </c>
-      <c r="N48" s="4" t="n"/>
+      <c r="N48" s="4" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="O48" s="4" t="n"/>
     </row>
     <row r="49">
@@ -3822,7 +4018,11 @@
 D: A generic tool puts no constraint on its inputs, so prompt guidance is the only barrier; a constrained alternative that validates its inputs would block these changes.</t>
         </is>
       </c>
-      <c r="N49" s="4" t="n"/>
+      <c r="N49" s="4" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="O49" s="4" t="n"/>
     </row>
     <row r="50">
@@ -3890,7 +4090,11 @@
 D: Error handling and escalation stay inside the subagent, so the coordinator still cannot observe failures or handle them consistently across cases.</t>
         </is>
       </c>
-      <c r="N50" s="4" t="n"/>
+      <c r="N50" s="4" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="O50" s="4" t="n"/>
     </row>
     <row r="51">
@@ -3958,7 +4162,11 @@
 D: /memory deals with the CLAUDE.md memory files that are loaded; it does not load an earlier session's conversation, which only --resume continues.</t>
         </is>
       </c>
-      <c r="N51" s="4" t="n"/>
+      <c r="N51" s="4" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="O51" s="4" t="n"/>
     </row>
     <row r="52">
@@ -4026,7 +4234,11 @@
 D: The guide states that keyword-sensitive system prompt wording can create unintended tool associations that override well-written tool descriptions.</t>
         </is>
       </c>
-      <c r="N52" s="4" t="n"/>
+      <c r="N52" s="4" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="O52" s="4" t="n"/>
     </row>
     <row r="53">
@@ -4094,7 +4306,11 @@
 D: Every message still goes through the full pipeline, and truncating output can harm complex cases; the guide's fix is dynamic subagent selection.</t>
         </is>
       </c>
-      <c r="N53" s="4" t="n"/>
+      <c r="N53" s="4" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="O53" s="4" t="n"/>
     </row>
     <row r="54">
@@ -4162,7 +4378,11 @@
 D: The guide names the description as the primary mechanism, and a new name keeps the minimal description with no example and no item ID edge case.</t>
         </is>
       </c>
-      <c r="N54" s="4" t="n"/>
+      <c r="N54" s="4" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="O54" s="4" t="n"/>
     </row>
     <row r="55">
@@ -4230,7 +4450,11 @@
 D: fork_session creates independent branches from a shared analysis baseline, so each divergent fix starts from the same analysis without influencing the other.</t>
         </is>
       </c>
-      <c r="N55" s="4" t="n"/>
+      <c r="N55" s="4" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="O55" s="4" t="n"/>
     </row>
     <row r="56">
@@ -4298,7 +4522,11 @@
 D: The details came from the customer's turns with the coordinator, not from a backend tool, and tool access does not give a subagent the coordinator's conversation history.</t>
         </is>
       </c>
-      <c r="N56" s="4" t="n"/>
+      <c r="N56" s="4" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="O56" s="4" t="n"/>
     </row>
     <row r="57">
@@ -4371,7 +4599,11 @@
 E: A generic error status hides the failure type, the attempted query and the partial results. The coordinator then cannot choose an appropriate recovery.</t>
         </is>
       </c>
-      <c r="N57" s="4" t="n"/>
+      <c r="N57" s="4" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="O57" s="4" t="n"/>
     </row>
     <row r="58">
@@ -4439,7 +4671,11 @@
 D: The customer's words lack the agent's findings, such as the payment-retry root cause, the refund amount and a recommended action, so the human agent must still re-investigate.</t>
         </is>
       </c>
-      <c r="N58" s="4" t="n"/>
+      <c r="N58" s="4" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="O58" s="4" t="n"/>
     </row>
     <row r="59">
@@ -4507,7 +4743,11 @@
 D: Claude can reason about the next action only when the tool result is appended to the conversation history. With the order data in context, Claude can move on to process_refund.</t>
         </is>
       </c>
-      <c r="N59" s="4" t="n"/>
+      <c r="N59" s="4" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="O59" s="4" t="n"/>
     </row>
     <row r="60">
@@ -4575,7 +4815,11 @@
 D: This avoids the format problem instead of normalizing the data, and escalating every return works against the 80%+ first-contact resolution target.</t>
         </is>
       </c>
-      <c r="N60" s="4" t="n"/>
+      <c r="N60" s="4" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="O60" s="4" t="n"/>
     </row>
     <row r="61">
@@ -4648,7 +4892,11 @@
 E: A human-readable description gives the agent the detail it needs to explain the problem and ask the customer for a corrected order number.</t>
         </is>
       </c>
-      <c r="N61" s="4" t="n"/>
+      <c r="N61" s="4" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
       <c r="O61" s="4" t="n"/>
     </row>
   </sheetData>

</xml_diff>